<commit_message>
📊 Actualizar METAS_MES_VU.xlsx — 08-04-2026, 12:09:05 p. m.
</commit_message>
<xml_diff>
--- a/datos/METAS_MES_VU.xlsx
+++ b/datos/METAS_MES_VU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df502c28020c5b60/Documentos/GIM/Proteccion Familiar/Estrategia/Estrategia 2026/3.Estrategia Comercial 2026/Dash board/Archivos 18032026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{1078BA19-444A-4B26-8041-59FC31F36ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2D12ADB-46B1-4357-806E-8D540D7268C1}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{AFBF8207-2148-4F4E-8E89-7A9E44F384BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5889879-F021-4651-B6F6-933C184265BE}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{628B001B-1F55-4D79-B631-1A95550BFD0D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{628B001B-1F55-4D79-B631-1A95550BFD0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta por lider" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Lider</t>
   </si>
@@ -66,6 +66,21 @@
   </si>
   <si>
     <t>Cantidad de Contratos</t>
+  </si>
+  <si>
+    <t>Humberto Barbiery</t>
+  </si>
+  <si>
+    <t>Patricia martinez</t>
+  </si>
+  <si>
+    <t>Sugey Vivas</t>
+  </si>
+  <si>
+    <t>Paula Garcia</t>
+  </si>
+  <si>
+    <t>Raul Bustos</t>
   </si>
 </sst>
 </file>
@@ -73,10 +88,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +114,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -108,7 +136,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -122,6 +150,13 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -130,19 +165,33 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
@@ -478,111 +527,171 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{239D0A04-0382-4C87-85C8-9F5AC02E0CEC}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="16.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
-        <v>26000000</v>
+      <c r="B3" s="13">
+        <v>35500000</v>
       </c>
       <c r="C3">
         <f>ROUND(B3/3200000,0)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="11">
         <v>0</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C7" si="0">ROUND(B4/3200000,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" s="1" t="s">
+        <f t="shared" ref="C4:C12" si="0">ROUND(B4/3200000,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
-        <v>26000000</v>
+      <c r="B5" s="13">
+        <v>35500000</v>
       </c>
       <c r="C5">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
-        <v>26000000</v>
+      <c r="B6" s="13">
+        <v>35500000</v>
       </c>
       <c r="C6">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4">
-        <v>26000000</v>
+      <c r="B7" s="13">
+        <v>35500000</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="12">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="10">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="11">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="10">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6">
-        <f>SUM(B3:B7)</f>
-        <v>104000000</v>
-      </c>
-      <c r="C8" s="6">
-        <f>SUM(C3:C7)</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" s="7"/>
-      <c r="B9" s="5"/>
-    </row>
-    <row r="10" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.45"/>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" s="1"/>
-      <c r="B11" s="5"/>
+      <c r="B13" s="8">
+        <f>SUM(B3:B12)</f>
+        <v>142000000</v>
+      </c>
+      <c r="C13" s="8">
+        <f>SUM(C3:C12)</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>